<commit_message>
frontend revamp and sensor panel
</commit_message>
<xml_diff>
--- a/Backend/app/ml/plant_care_database.xlsx
+++ b/Backend/app/ml/plant_care_database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\missc\EEE_ES\Backend\app\ml\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF9A59B4-5A44-4A39-AC88-F28ADE07C3FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90DCCBB8-AAEA-437C-ADA9-BD4016234253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="8904" xr2:uid="{519D503D-ED95-41E0-9E5F-9F40720A94E6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="13">
   <si>
     <t>Plant Name</t>
   </si>
@@ -44,18 +44,9 @@
     <t>Light Requirement</t>
   </si>
   <si>
-    <t>Medium indirect</t>
-  </si>
-  <si>
     <t>Low</t>
   </si>
   <si>
-    <t>Medium  indirect</t>
-  </si>
-  <si>
-    <t>Bright direct</t>
-  </si>
-  <si>
     <t>Moisture Requirement</t>
   </si>
   <si>
@@ -81,6 +72,9 @@
   </si>
   <si>
     <t>salvia_officinales</t>
+  </si>
+  <si>
+    <t>Bright Direct</t>
   </si>
 </sst>
 </file>
@@ -468,73 +462,73 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
         <v>5</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
         <v>5</v>
-      </c>
-      <c r="C6" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
         <v>5</v>
-      </c>
-      <c r="C7" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>